<commit_message>
Update speaking opportunities: open only, add Encore targets, topics and strategy
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181Kt2UaK9uGnQWm9d9jutU
</commit_message>
<xml_diff>
--- a/outbox/speaking-opportunities-2026-10-19.xlsx
+++ b/outbox/speaking-opportunities-2026-10-19.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Opportunities" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Encore Topics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Open Opportunities'!$A$1:$K$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Open Opportunities'!$A$1:$K$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -635,7 +637,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Seramount (formerly Diversity Best Practices) events call for speakers 2027</t>
+          <t>Seramount events call for speakers 2027</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -692,42 +694,42 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Agent Conference NYC 2027</t>
+          <t>Women's Leadership Conference 2027: Seasons of Her</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>AI systems</t>
+          <t>Encore / identity</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>May 17-18, 2027</t>
+          <t>Apr 30, 2027</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Rolling, no deadline</t>
+          <t>Not stated on page</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>New York Hilton Midtown, in person</t>
+          <t>Southern Oregon, in person</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Keynote (50 min): modest honorarium. Lightning talk (15 min): volunteer</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Theme 'Agentic Enterprises' fits her working agent systems. Product pitches banned; must be practitioner story. Best venue for the AI-architect angle.</t>
+          <t>Best Encore fit found: theme is the seasons of a woman's life and leadership. Needs a 2-3 minute intro video, session description and bio.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Draft a practitioner-case proposal; submit via portal</t>
+          <t>Record the intro video; submit a lightning talk or keynote</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -737,7 +739,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>https://www.agentconference.com/call-for-proposals</t>
+          <t>https://womensleadership.co/conference-2027/</t>
         </is>
       </c>
     </row>
@@ -749,52 +751,52 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>WorkHuman Live Nashville 2027</t>
+          <t>Women Thrive Summit 2027</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Executive comms / AI</t>
+          <t>Encore</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Apr 26-29, 2027</t>
+          <t>Mar 15-19, 2027</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Rolling, open year-round</t>
+          <t>No deadline stated; waitlist form</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Nashville, in person</t>
+          <t>Virtual</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Speakers pay an 'investment' (amount not stated)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Already in tracker. Video sample required by the form.</t>
+          <t>Footage and exposure; 30 percent of slots reserved for first-time speakers. Pay-to-speak: only if the fee is small.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Record a 2-3 minute sample (recording from #1 or #2 can serve)</t>
+          <t>Ask for the fee before committing</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Blocked on video sample</t>
+          <t>Open, pay-to-speak</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>memory/projects/speaking-targets.md</t>
+          <t>https://womenthrivesummit.com/speaker/</t>
         </is>
       </c>
     </row>
@@ -806,52 +808,52 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ATD South Florida chapter speaker program</t>
+          <t>Black Enterprise Women of Power Summit 2027</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>AI systems / exec comms</t>
+          <t>Encore / legacy</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Mar 7-11, 2027</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Rolling</t>
+          <t>Not read; page links to a 'Become a Speaker' page</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>South Florida</t>
+          <t>Bellagio, Las Vegas</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Not indicated (chapters rarely pay)</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Local, easy first yes; a good source of footage.</t>
+          <t>Large audience of Black women professionals; fits Legacy Salon positioning.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Approve and send the existing pitch</t>
+          <t>Read blackenterprise.com/wpsbecomeaspeaker and confirm process</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Needs verification</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>outbox/speaking-pitch-atd-south-florida.md</t>
+          <t>https://www.blackenterprise.com/women-of-power-2027/</t>
         </is>
       </c>
     </row>
@@ -863,52 +865,52 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ATD Central Florida (ATDCFL)</t>
+          <t>Create &amp; Cultivate Festival, Los Angeles</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>AI systems / exec comms</t>
+          <t>Encore / lifestyle</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Sep 25-26, 2027</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Rolling (verify live page)</t>
+          <t>No public speaker application found</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Orlando</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Not indicated</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Same talk as ATD South Florida.</t>
+          <t>Target stage. Site shows only sponsor and partner inquiries and an application-or-referral Supper Club (Miami). See Strategy tab.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Draft pitch (not yet written)</t>
+          <t>Follow the Create &amp; Cultivate path in the Strategy tab</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Not yet pitched</t>
+          <t>Long-term target</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>memory/projects/speaking-targets.md</t>
+          <t>https://www.createcultivate.com</t>
         </is>
       </c>
     </row>
@@ -920,52 +922,52 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>How to Be Awesome at Your Job (podcast, Pete Mockaitis)</t>
+          <t>Agent Conference NYC 2027</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Exec comms</t>
+          <t>AI systems</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>May 17-18, 2027</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Rolling</t>
+          <t>Rolling, no deadline</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>New York Hilton Midtown, in person</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Unpaid (guest booking)</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Audience building and clips; not paid.</t>
+          <t>Theme 'Agentic Enterprises' fits her working agent systems. Product pitches banned; must be practitioner story. Best venue for the AI-architect angle.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Approve and send the existing pitch</t>
+          <t>Draft a practitioner-case proposal; submit via portal</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>outbox/speaking-pitch-how-to-be-awesome-at-your-job.md</t>
+          <t>https://www.agentconference.com/call-for-proposals</t>
         </is>
       </c>
     </row>
@@ -977,27 +979,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ACMP general inquiry (2028 and chapters)</t>
+          <t>WorkHuman Live Nashville 2027</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>AI systems</t>
+          <t>Executive comms / AI</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Future</t>
+          <t>Apr 26-29, 2027</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2027 call closed Sep 30, 2026</t>
+          <t>Rolling, open year-round</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Various</t>
+          <t>Nashville, in person</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1007,22 +1009,22 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Best topical fit (AI applications in change management track). Ask about 2028 and chapter and webinar slots.</t>
+          <t>Already in tracker. Video sample required by the form.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Approve the existing inquiry</t>
+          <t>Record a 2-3 minute sample (recording from #1 or #2 can serve)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Draft ready</t>
+          <t>Blocked on video sample</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>outbox/speaking-pitch-acmp-inquiry.md</t>
+          <t>memory/projects/speaking-targets.md</t>
         </is>
       </c>
     </row>
@@ -1034,52 +1036,52 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Women's Leadership and Empowerment Conference WLEC2027</t>
+          <t>ATD South Florida chapter speaker program</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Encore / identity</t>
+          <t>AI systems / exec comms</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Mar 1-3, 2027</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Dec 25, 2026 (rolling, may close earlier)</t>
+          <t>Rolling</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Bangkok, Thailand</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Not stated; likely fee-based</t>
+          <t>Not indicated (chapters rarely pay)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Academic-style, travel-heavy and unlikely to pay. Low priority.</t>
+          <t>Local, easy first yes; a good source of footage.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Skip unless a funded travel plan exists</t>
+          <t>Approve and send the existing pitch</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Low priority</t>
+          <t>Draft ready</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>https://www.wleconference.org/call-for-papers.html</t>
+          <t>outbox/speaking-pitch-atd-south-florida.md</t>
         </is>
       </c>
     </row>
@@ -1091,52 +1093,52 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>South Florida Women in Tech (Sessionize)</t>
+          <t>ATD Central Florida (ATDCFL)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>AI systems</t>
+          <t>AI systems / exec comms</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Nov 12 and Dec 10, 2026</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Nov 27, 2026</t>
+          <t>Rolling (verify live page)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Orlando</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Not indicated</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Topics are developer-oriented; poor fit.</t>
+          <t>Same talk as ATD South Florida.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Draft pitch (not yet written)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Poor fit</t>
+          <t>Not yet pitched</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>https://sessionize.com/south-florida-women-in-tech/</t>
+          <t>memory/projects/speaking-targets.md</t>
         </is>
       </c>
     </row>
@@ -1148,52 +1150,52 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>The Conference for Women (Central PA)</t>
+          <t>How to Be Awesome at Your Job (podcast, Pete Mockaitis)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Encore</t>
+          <t>Exec comms</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2027 date TBD</t>
+          <t>Ongoing</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>No deadline stated</t>
+          <t>Rolling</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Camp Hill, PA area</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Unpaid (pro bono stated)</t>
+          <t>Unpaid (guest booking)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Women's audience but unpaid and far away.</t>
+          <t>Audience building and clips; not paid.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Skip unless travel and exposure justify it</t>
+          <t>Approve and send the existing pitch</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Low priority</t>
+          <t>Draft ready</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>https://www.conference4women.com/submit-a-proposal</t>
+          <t>outbox/speaking-pitch-how-to-be-awesome-at-your-job.md</t>
         </is>
       </c>
     </row>
@@ -1205,52 +1207,52 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Internal Comms Conference Manchester</t>
+          <t>Women's Leadership and Empowerment Conference WLEC2027</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Exec comms</t>
+          <t>Encore / identity</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Jan 21, 2027</t>
+          <t>Mar 1-3, 2027</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>No call for speakers posted</t>
+          <t>Dec 25, 2026 (rolling, may close earlier)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Manchester, UK</t>
+          <t>Bangkok, Thailand</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Not stated; likely fee-based</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Internal communications audience. Direct inquiry only: partner@internalconference.com.</t>
+          <t>Academic-style, travel-heavy and unlikely to pay. Low priority.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Optional email inquiry</t>
+          <t>Skip unless a funded travel plan exists</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Direct inquiry only</t>
+          <t>Low priority</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>https://internalconference.com/</t>
+          <t>https://www.wleconference.org/call-for-papers.html</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1264,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>SHRM AI+HI Project 2027</t>
+          <t>South Florida Women in Tech (Sessionize)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1272,17 +1274,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Nov 12 and Dec 10, 2026</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Not open (notify-me stage)</t>
+          <t>Nov 27, 2026</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1292,22 +1294,22 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Direct fit with AI and HR leaders.</t>
+          <t>Topics are developer-oriented; poor fit.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Sign up for notification if not done</t>
+          <t>Skip</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Poor fit</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>memory/projects/speaking-targets.md</t>
+          <t>https://sessionize.com/south-florida-women-in-tech/</t>
         </is>
       </c>
     </row>
@@ -1319,52 +1321,52 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>HR Florida 2027 (SHRM Florida)</t>
+          <t>The Conference for Women (Central PA)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Exec comms / AI</t>
+          <t>Encore</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Likely late summer 2027</t>
+          <t>2027 date TBD</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed; a 2027 proposal survey link appeared in search</t>
+          <t>No deadline stated</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Camp Hill, PA area</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Unpaid (pro bono stated)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Previous cycle's proposals closed July 2026.</t>
+          <t>Women's audience but unpaid and far away.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Verify live page and whether a 2027 call is open</t>
+          <t>Skip unless travel and exposure justify it</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Needs verification</t>
+          <t>Low priority</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Search result only, not read</t>
+          <t>https://www.conference4women.com/submit-a-proposal</t>
         </is>
       </c>
     </row>
@@ -1376,27 +1378,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>ACMP 2027 (Change Denver May 1-4; Global Connect Jun 8-10; webinars)</t>
+          <t>Internal Comms Conference Manchester</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>AI systems</t>
+          <t>Exec comms</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>May-Jun 2027</t>
+          <t>Jan 21, 2027</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Closed Sep 30, 2026</t>
+          <t>No call for speakers posted</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Aurora CO; virtual</t>
+          <t>Manchester, UK</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1406,22 +1408,22 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Missed. Correction: the Oct 16 ACMP deadline in my earlier note was wrong; the real deadline was Sep 30.</t>
+          <t>Internal communications audience. Direct inquiry only: partner@internalconference.com.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Optional email inquiry</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Direct inquiry only</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>https://www.acmpglobal.org/page/2027-call-for-speakers</t>
+          <t>https://internalconference.com/</t>
         </is>
       </c>
     </row>
@@ -1433,57 +1435,114 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Women in Payments USA 2027</t>
+          <t>SHRM AI+HI Project 2027</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Encore</t>
+          <t>AI systems</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Not open (notify-me stage)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Direct fit with AI and HR leaders.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Sign up for notification if not done</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>memory/projects/speaking-targets.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>HR Florida 2027 (SHRM Florida)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Exec comms / AI</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Likely late summer 2027</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed; a 2027 proposal survey link appeared in search</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Florida</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Speakers pay for a pass</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Closed and pay-to-play.</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>https://info.womeninpayments.org/call-for-speakers-usa-2027-registration-page</t>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Previous cycle's proposals closed July 2026.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Verify live page and whether a 2027 call is open</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Needs verification</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Search result only, not read</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K18"/>
+  <autoFilter ref="A1:K19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1524,7 +1583,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Coverage is not exhaustive. Search returned few primary pages for executive communications and Encore-themed events; Ragan, PRSA and IABC 2027 calls were not confirmed and are not listed.</t>
+          <t>Closed calls were removed on Oct 19, 2026 at Tonya's request (ACMP 2027, Women in Payments). Unpaid is acceptable to Tonya for building a track record and footage. Women Professionals Wellness requires a clinical practice and Empowered Women in Wellness dates are in 2026 and past; both left out. Coverage is not exhaustive. Search returned few primary pages for executive communications and Encore-themed events; Ragan, PRSA and IABC 2027 calls were not confirmed and are not listed.</t>
         </is>
       </c>
     </row>
@@ -1532,6 +1591,318 @@
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Entreprenista and Beyond Cowork details come from Tonya and her inbox; dates and fees are not verified here.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Talk title (working)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Core idea</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Audience</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Proof to build</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Your Encore Era</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Midlife as a chosen chapter with a point of view, not a comeback. Replaces the overused reinvention frame.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Women 40+ and 50+ events</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Entreprenista workshop recording</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>The Room Where Women Are Heard</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Why intimate, story-led gatherings build trust faster than networking events; the Salon dinner model.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Women entrepreneurs, community builders</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Your first Salon Dinner (Mar 6, 2026, 12 women); get one guest quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Legacy as a Living Practice</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Building assets, stories and relationships your family and community can inherit.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Black women, wealth and legacy events</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Salon Series</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Presence After 50</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Style, voice and visibility as strategy; being seen on purpose.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Lifestyle and women-in-business festivals</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Short video clips</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Tell It on Purpose</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Using your own story as a brand asset, from 20 years of storytelling work.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Creators, founders, career pivoters</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Substack and LinkedIn posts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Quiet Systems, Louder Life</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>How a small set of AI tools buys back time for a woman building a brand. Bridges Encore to your AI-systems credibility.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Women founders and creators</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Your own weekly operating system, shown live</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Capture footage of the Entreprenista workshop and the Nov 19 summit session. Cut a 2-3 minute sample reel. Several applications (Seasons of Her, WorkHuman Live) require video.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Nov to Dec 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Set a cadence of one stage a month: one unpaid talk, one clip posted, one new pitch each week. Start with ATD South Florida, the Seasons of Her call and Seramount.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Monthly from Nov 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Use your Salon dinners as an owned stage: invite one speaker-adjacent guest each time and record permissioned highlights.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Create &amp; Cultivate publishes no speaker application that I could find. Realistic routes: attend, build a relationship with their events team, apply to the application-only Supper Club, and pitch the 2028 festival once you have a reel and 3 to 5 stages behind you. These routes are my inference, not confirmed by their site.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Attend or apply in 2027; pitch 2028</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Ask each organizer for a testimonial and a headshot-on-stage photo; add them to a one-page speaker sheet.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>After each talk</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Review quarterly: stages completed, footage captured, inbound invitations. Move to paid asks after 4 to 6 recorded talks.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2027 review</t>
         </is>
       </c>
     </row>

</xml_diff>